<commit_message>
02 febrero 2022 v1
</commit_message>
<xml_diff>
--- a/_downloads/219fb1d9309965b5498bc9255adc60a7/Ejemplo Flujo de Efectivo H&M.xlsx
+++ b/_downloads/219fb1d9309965b5498bc9255adc60a7/Ejemplo Flujo de Efectivo H&M.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\UNAL\ADMINISTRACIÓN FINANCIERA\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E06B6999-5154-4DFD-A13C-CC7253FC04C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E40B89F2-2167-4869-9302-9DBAD1069848}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{96756974-1267-4C41-A3A6-DE3697CF134B}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="107">
   <si>
     <t>H&amp;M HENNES &amp; MAURITZ COLOMBIA S.A.S</t>
   </si>
@@ -513,10 +513,19 @@
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -531,23 +540,17 @@
     <xf numFmtId="165" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -555,14 +558,11 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -906,8 +906,8 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="21"/>
-      <c r="B5" s="22"/>
+      <c r="A5" s="11"/>
+      <c r="B5" s="21"/>
       <c r="C5" s="2">
         <v>2017</v>
       </c>
@@ -922,10 +922,10 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="14"/>
+      <c r="B6" s="17"/>
       <c r="C6" s="4">
         <v>61719652</v>
       </c>
@@ -940,10 +940,10 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="14"/>
+      <c r="B7" s="17"/>
       <c r="C7" s="4">
         <v>16010669</v>
       </c>
@@ -958,10 +958,10 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="14"/>
+      <c r="B8" s="17"/>
       <c r="C8" s="4">
         <v>41791255</v>
       </c>
@@ -976,10 +976,10 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="14"/>
+      <c r="B9" s="17"/>
       <c r="C9" s="4">
         <v>1485552</v>
       </c>
@@ -990,20 +990,20 @@
       <c r="F9" s="4"/>
     </row>
     <row r="10" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="14"/>
+      <c r="B10" s="17"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
     </row>
     <row r="11" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="13" t="s">
+      <c r="A11" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="14"/>
+      <c r="B11" s="17"/>
       <c r="C11" s="4">
         <v>2669096</v>
       </c>
@@ -1018,10 +1018,10 @@
       </c>
     </row>
     <row r="12" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="16"/>
+      <c r="B12" s="19"/>
       <c r="C12" s="5">
         <f>SUM(C6:C11)</f>
         <v>123676224</v>
@@ -1040,20 +1040,20 @@
       </c>
     </row>
     <row r="13" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="14"/>
+      <c r="B13" s="17"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
     </row>
     <row r="14" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A14" s="13" t="s">
+      <c r="A14" s="16" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="14"/>
+      <c r="B14" s="17"/>
       <c r="C14" s="4">
         <v>57777446</v>
       </c>
@@ -1068,50 +1068,50 @@
       </c>
     </row>
     <row r="15" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="13" t="s">
+      <c r="A15" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="14"/>
+      <c r="B15" s="17"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
     </row>
     <row r="16" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A16" s="13" t="s">
+      <c r="A16" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="14"/>
+      <c r="B16" s="17"/>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
     </row>
     <row r="17" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="14"/>
+      <c r="B17" s="17"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
     </row>
     <row r="18" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A18" s="13" t="s">
+      <c r="A18" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="14"/>
+      <c r="B18" s="17"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
     </row>
     <row r="19" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A19" s="13" t="s">
+      <c r="A19" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="14"/>
+      <c r="B19" s="17"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4">
@@ -1122,30 +1122,30 @@
       </c>
     </row>
     <row r="20" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="14"/>
+      <c r="B20" s="17"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
     </row>
     <row r="21" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A21" s="13" t="s">
+      <c r="A21" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="14"/>
+      <c r="B21" s="17"/>
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
     </row>
     <row r="22" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="15" t="s">
+      <c r="A22" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="16"/>
+      <c r="B22" s="19"/>
       <c r="C22" s="5">
         <f>SUM(C13:C21)</f>
         <v>57777446</v>
@@ -1164,10 +1164,10 @@
       </c>
     </row>
     <row r="23" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="15" t="s">
+      <c r="A23" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B23" s="16"/>
+      <c r="B23" s="19"/>
       <c r="C23" s="5">
         <f>+C12+C22</f>
         <v>181453670</v>
@@ -1186,10 +1186,10 @@
       </c>
     </row>
     <row r="24" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A24" s="13" t="s">
+      <c r="A24" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B24" s="14"/>
+      <c r="B24" s="17"/>
       <c r="C24" s="4">
         <v>920670</v>
       </c>
@@ -1204,10 +1204,10 @@
       </c>
     </row>
     <row r="25" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A25" s="13" t="s">
+      <c r="A25" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="14"/>
+      <c r="B25" s="17"/>
       <c r="C25" s="4">
         <v>610000</v>
       </c>
@@ -1218,10 +1218,10 @@
       <c r="F25" s="4"/>
     </row>
     <row r="26" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A26" s="13" t="s">
+      <c r="A26" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="B26" s="14"/>
+      <c r="B26" s="17"/>
       <c r="C26" s="4">
         <v>116865783</v>
       </c>
@@ -1236,10 +1236,10 @@
       </c>
     </row>
     <row r="27" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A27" s="13" t="s">
+      <c r="A27" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="B27" s="14"/>
+      <c r="B27" s="17"/>
       <c r="C27" s="4">
         <v>588184</v>
       </c>
@@ -1254,10 +1254,10 @@
       </c>
     </row>
     <row r="28" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A28" s="13" t="s">
+      <c r="A28" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="B28" s="14"/>
+      <c r="B28" s="17"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
       <c r="E28" s="4">
@@ -1268,10 +1268,10 @@
       </c>
     </row>
     <row r="29" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A29" s="13" t="s">
+      <c r="A29" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="B29" s="14"/>
+      <c r="B29" s="17"/>
       <c r="C29" s="4">
         <v>831606</v>
       </c>
@@ -1284,10 +1284,10 @@
       </c>
     </row>
     <row r="30" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A30" s="15" t="s">
+      <c r="A30" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="B30" s="16"/>
+      <c r="B30" s="19"/>
       <c r="C30" s="5">
         <f>SUM(C24:C29)</f>
         <v>119816243</v>
@@ -1306,30 +1306,30 @@
       </c>
     </row>
     <row r="31" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A31" s="13" t="s">
+      <c r="A31" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="B31" s="14"/>
+      <c r="B31" s="17"/>
       <c r="C31" s="4"/>
       <c r="D31" s="4"/>
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
     </row>
     <row r="32" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A32" s="13" t="s">
+      <c r="A32" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="B32" s="14"/>
+      <c r="B32" s="17"/>
       <c r="C32" s="4"/>
       <c r="D32" s="4"/>
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
     </row>
     <row r="33" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A33" s="13" t="s">
+      <c r="A33" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="B33" s="14"/>
+      <c r="B33" s="17"/>
       <c r="C33" s="4">
         <v>55482500</v>
       </c>
@@ -1342,30 +1342,30 @@
       </c>
     </row>
     <row r="34" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A34" s="13" t="s">
+      <c r="A34" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="B34" s="14"/>
+      <c r="B34" s="17"/>
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
     </row>
     <row r="35" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A35" s="13" t="s">
+      <c r="A35" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="B35" s="14"/>
+      <c r="B35" s="17"/>
       <c r="C35" s="4"/>
       <c r="D35" s="4"/>
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
     </row>
     <row r="36" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A36" s="13" t="s">
+      <c r="A36" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="B36" s="14"/>
+      <c r="B36" s="17"/>
       <c r="C36" s="4"/>
       <c r="D36" s="4">
         <v>103658589</v>
@@ -1378,10 +1378,10 @@
       </c>
     </row>
     <row r="37" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A37" s="13" t="s">
+      <c r="A37" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="B37" s="14"/>
+      <c r="B37" s="17"/>
       <c r="C37" s="4"/>
       <c r="D37" s="4">
         <v>1324193</v>
@@ -1394,10 +1394,10 @@
       </c>
     </row>
     <row r="38" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A38" s="15" t="s">
+      <c r="A38" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="B38" s="16"/>
+      <c r="B38" s="19"/>
       <c r="C38" s="5">
         <f>SUM(C31:C37)</f>
         <v>55482500</v>
@@ -1416,10 +1416,10 @@
       </c>
     </row>
     <row r="39" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A39" s="15" t="s">
+      <c r="A39" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="B39" s="16"/>
+      <c r="B39" s="19"/>
       <c r="C39" s="5">
         <f>+C30+C38</f>
         <v>175298743</v>
@@ -1438,10 +1438,10 @@
       </c>
     </row>
     <row r="40" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A40" s="13" t="s">
+      <c r="A40" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="B40" s="14"/>
+      <c r="B40" s="17"/>
       <c r="C40" s="4">
         <v>2521750</v>
       </c>
@@ -1456,10 +1456,10 @@
       </c>
     </row>
     <row r="41" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A41" s="13" t="s">
+      <c r="A41" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="B41" s="14"/>
+      <c r="B41" s="17"/>
       <c r="C41" s="4">
         <v>22065750</v>
       </c>
@@ -1474,10 +1474,10 @@
       </c>
     </row>
     <row r="42" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A42" s="13" t="s">
+      <c r="A42" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="B42" s="14"/>
+      <c r="B42" s="17"/>
       <c r="C42" s="4">
         <v>-18432573</v>
       </c>
@@ -1492,10 +1492,10 @@
       </c>
     </row>
     <row r="43" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A43" s="15" t="s">
+      <c r="A43" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="B43" s="16"/>
+      <c r="B43" s="19"/>
       <c r="C43" s="5">
         <f>SUM(C40:C42)</f>
         <v>6154927</v>
@@ -1514,10 +1514,10 @@
       </c>
     </row>
     <row r="44" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A44" s="15" t="s">
+      <c r="A44" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="B44" s="16"/>
+      <c r="B44" s="19"/>
       <c r="C44" s="5">
         <f>+C39+C43</f>
         <v>181453670</v>
@@ -1536,16 +1536,16 @@
       </c>
     </row>
     <row r="45" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A45" s="25"/>
-      <c r="B45" s="25"/>
+      <c r="A45" s="13"/>
+      <c r="B45" s="13"/>
     </row>
     <row r="46" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A46" s="25"/>
-      <c r="B46" s="25"/>
+      <c r="A46" s="13"/>
+      <c r="B46" s="13"/>
     </row>
     <row r="47" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A47" s="25"/>
-      <c r="B47" s="26"/>
+      <c r="A47" s="13"/>
+      <c r="B47" s="20"/>
       <c r="C47" s="2">
         <v>2017</v>
       </c>
@@ -1560,10 +1560,10 @@
       </c>
     </row>
     <row r="48" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A48" s="13" t="s">
+      <c r="A48" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="B48" s="14"/>
+      <c r="B48" s="17"/>
       <c r="C48" s="4">
         <v>95221493</v>
       </c>
@@ -1577,11 +1577,11 @@
         <v>209537978</v>
       </c>
     </row>
-    <row r="49" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A49" s="13" t="s">
+    <row r="49" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A49" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="B49" s="14"/>
+      <c r="B49" s="17"/>
       <c r="C49" s="4">
         <v>48837338</v>
       </c>
@@ -1595,11 +1595,11 @@
         <v>107450900</v>
       </c>
     </row>
-    <row r="50" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A50" s="15" t="s">
+    <row r="50" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A50" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="B50" s="16"/>
+      <c r="B50" s="19"/>
       <c r="C50" s="5">
         <f>+C48-C49</f>
         <v>46384155</v>
@@ -1617,11 +1617,11 @@
         <v>102087078</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A51" s="13" t="s">
+    <row r="51" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A51" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="B51" s="14"/>
+      <c r="B51" s="17"/>
       <c r="C51" s="4">
         <v>5388102</v>
       </c>
@@ -1629,11 +1629,11 @@
       <c r="E51" s="4"/>
       <c r="F51" s="4"/>
     </row>
-    <row r="52" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A52" s="13" t="s">
+    <row r="52" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A52" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="B52" s="14"/>
+      <c r="B52" s="17"/>
       <c r="C52" s="4">
         <v>41445847</v>
       </c>
@@ -1645,11 +1645,11 @@
         <v>66786465</v>
       </c>
     </row>
-    <row r="53" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A53" s="13" t="s">
+    <row r="53" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A53" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="B53" s="14"/>
+      <c r="B53" s="17"/>
       <c r="C53" s="4">
         <v>19209605</v>
       </c>
@@ -1663,11 +1663,11 @@
         <v>11467772</v>
       </c>
     </row>
-    <row r="54" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A54" s="13" t="s">
+    <row r="54" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A54" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="B54" s="14"/>
+      <c r="B54" s="17"/>
       <c r="C54" s="4">
         <v>627842</v>
       </c>
@@ -1677,11 +1677,11 @@
       <c r="E54" s="4"/>
       <c r="F54" s="4"/>
     </row>
-    <row r="55" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A55" s="13" t="s">
+    <row r="55" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A55" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="B55" s="14"/>
+      <c r="B55" s="17"/>
       <c r="C55" s="4"/>
       <c r="D55" s="4">
         <v>-3781821</v>
@@ -1693,11 +1693,11 @@
         <v>-1879639</v>
       </c>
     </row>
-    <row r="56" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A56" s="15" t="s">
+    <row r="56" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A56" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="B56" s="16"/>
+      <c r="B56" s="19"/>
       <c r="C56" s="5">
         <f>+C50+C51-C52-C53-C54+C55</f>
         <v>-9511037</v>
@@ -1714,12 +1714,13 @@
         <f>+F50+F51-F52-F53-F54+F55</f>
         <v>21953202</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A57" s="13" t="s">
+      <c r="G56" s="7"/>
+    </row>
+    <row r="57" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A57" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="B57" s="14"/>
+      <c r="B57" s="17"/>
       <c r="C57" s="4">
         <v>312884</v>
       </c>
@@ -1733,11 +1734,11 @@
         <v>273447</v>
       </c>
     </row>
-    <row r="58" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A58" s="13" t="s">
+    <row r="58" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A58" s="16" t="s">
         <v>52</v>
       </c>
-      <c r="B58" s="14"/>
+      <c r="B58" s="17"/>
       <c r="C58" s="4">
         <v>7196584</v>
       </c>
@@ -1751,11 +1752,11 @@
         <v>5544644</v>
       </c>
     </row>
-    <row r="59" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A59" s="15" t="s">
+    <row r="59" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A59" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="B59" s="16"/>
+      <c r="B59" s="19"/>
       <c r="C59" s="5">
         <f>+C56+C57-C58</f>
         <v>-16394737</v>
@@ -1773,11 +1774,11 @@
         <v>16682005</v>
       </c>
     </row>
-    <row r="60" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A60" s="13" t="s">
+    <row r="60" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A60" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="B60" s="14"/>
+      <c r="B60" s="17"/>
       <c r="C60" s="4">
         <v>0</v>
       </c>
@@ -1791,11 +1792,11 @@
         <v>6524343</v>
       </c>
     </row>
-    <row r="61" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A61" s="15" t="s">
+    <row r="61" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A61" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="B61" s="16"/>
+      <c r="B61" s="19"/>
       <c r="C61" s="5">
         <f>+C59-C60</f>
         <v>-16394737</v>
@@ -1813,15 +1814,15 @@
         <v>10157662</v>
       </c>
     </row>
-    <row r="62" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A62" s="25"/>
-      <c r="B62" s="25"/>
-    </row>
-    <row r="63" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A63" s="19" t="s">
+    <row r="62" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A62" s="13"/>
+      <c r="B62" s="13"/>
+    </row>
+    <row r="63" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A63" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="B63" s="20"/>
+      <c r="B63" s="15"/>
       <c r="C63" s="4">
         <v>3882481</v>
       </c>
@@ -1835,11 +1836,11 @@
         <v>18286619</v>
       </c>
     </row>
-    <row r="64" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A64" s="13" t="s">
+    <row r="64" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="A64" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="B64" s="14"/>
+      <c r="B64" s="17"/>
       <c r="C64" s="5">
         <f>+C56+C63</f>
         <v>-5628556</v>
@@ -1871,13 +1872,11 @@
       </c>
     </row>
     <row r="68" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A68" s="21" t="s">
-        <v>57</v>
-      </c>
-      <c r="B68" s="11" t="s">
+      <c r="A68" s="11"/>
+      <c r="B68" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="C68" s="12"/>
+      <c r="C68" s="23"/>
       <c r="D68" s="4">
         <f>+D61</f>
         <v>-2861832</v>
@@ -1893,11 +1892,11 @@
       <c r="G68" s="7"/>
     </row>
     <row r="69" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A69" s="21"/>
-      <c r="B69" s="23" t="s">
+      <c r="A69" s="11"/>
+      <c r="B69" s="24" t="s">
         <v>98</v>
       </c>
-      <c r="C69" s="24"/>
+      <c r="C69" s="25"/>
       <c r="D69" s="4">
         <f>+D63</f>
         <v>8343094</v>
@@ -1913,11 +1912,11 @@
       <c r="G69" s="7"/>
     </row>
     <row r="70" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A70" s="21"/>
-      <c r="B70" s="19" t="s">
+      <c r="A70" s="11"/>
+      <c r="B70" s="14" t="s">
         <v>96</v>
       </c>
-      <c r="C70" s="20"/>
+      <c r="C70" s="15"/>
       <c r="D70" s="4">
         <f>-D57</f>
         <v>-481784</v>
@@ -1932,11 +1931,11 @@
       </c>
     </row>
     <row r="71" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A71" s="21"/>
-      <c r="B71" s="19" t="s">
+      <c r="A71" s="11"/>
+      <c r="B71" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="C71" s="20"/>
+      <c r="C71" s="15"/>
       <c r="D71" s="4">
         <f>+D58</f>
         <v>6052503</v>
@@ -1951,13 +1950,13 @@
       </c>
     </row>
     <row r="72" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A72" s="21" t="s">
+      <c r="A72" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="B72" s="19" t="s">
+      <c r="B72" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="C72" s="20"/>
+      <c r="C72" s="15"/>
       <c r="D72" s="4">
         <f t="shared" ref="D72:F73" si="11">+C7-D7</f>
         <v>-1038000</v>
@@ -1972,11 +1971,11 @@
       </c>
     </row>
     <row r="73" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A73" s="21"/>
-      <c r="B73" s="19" t="s">
+      <c r="A73" s="11"/>
+      <c r="B73" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="C73" s="20"/>
+      <c r="C73" s="15"/>
       <c r="D73" s="4">
         <f t="shared" si="11"/>
         <v>13631656</v>
@@ -1991,11 +1990,11 @@
       </c>
     </row>
     <row r="74" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A74" s="21"/>
-      <c r="B74" s="19" t="s">
+      <c r="A74" s="11"/>
+      <c r="B74" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="C74" s="20"/>
+      <c r="C74" s="15"/>
       <c r="D74" s="4">
         <f>+D26-C26</f>
         <v>-56262023</v>
@@ -2010,13 +2009,13 @@
       </c>
     </row>
     <row r="75" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A75" s="21" t="s">
+      <c r="A75" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="B75" s="19" t="s">
+      <c r="B75" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="C75" s="20"/>
+      <c r="C75" s="15"/>
       <c r="D75" s="4">
         <f t="shared" ref="D75:F77" si="12">+C9-D9</f>
         <v>1249464</v>
@@ -2031,11 +2030,11 @@
       </c>
     </row>
     <row r="76" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A76" s="21"/>
-      <c r="B76" s="19" t="s">
+      <c r="A76" s="11"/>
+      <c r="B76" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="C76" s="20"/>
+      <c r="C76" s="15"/>
       <c r="D76" s="4">
         <f t="shared" si="12"/>
         <v>0</v>
@@ -2050,11 +2049,11 @@
       </c>
     </row>
     <row r="77" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A77" s="21"/>
-      <c r="B77" s="19" t="s">
+      <c r="A77" s="11"/>
+      <c r="B77" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="C77" s="20"/>
+      <c r="C77" s="15"/>
       <c r="D77" s="4">
         <f t="shared" si="12"/>
         <v>2607609</v>
@@ -2069,13 +2068,13 @@
       </c>
     </row>
     <row r="78" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A78" s="21" t="s">
+      <c r="A78" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="B78" s="19" t="s">
+      <c r="B78" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="C78" s="20"/>
+      <c r="C78" s="15"/>
       <c r="D78" s="4">
         <f t="shared" ref="D78:F79" si="13">+D24-C24</f>
         <v>-142685</v>
@@ -2088,16 +2087,16 @@
         <f t="shared" si="13"/>
         <v>-88511</v>
       </c>
-      <c r="G78" s="27" t="s">
+      <c r="G78" s="12" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="79" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A79" s="21"/>
-      <c r="B79" s="19" t="s">
+      <c r="A79" s="11"/>
+      <c r="B79" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="C79" s="20"/>
+      <c r="C79" s="15"/>
       <c r="D79" s="4">
         <f t="shared" si="13"/>
         <v>2972232</v>
@@ -2110,14 +2109,14 @@
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
-      <c r="G79" s="27"/>
+      <c r="G79" s="12"/>
     </row>
     <row r="80" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A80" s="21"/>
-      <c r="B80" s="19" t="s">
+      <c r="A80" s="11"/>
+      <c r="B80" s="14" t="s">
         <v>64</v>
       </c>
-      <c r="C80" s="20"/>
+      <c r="C80" s="15"/>
       <c r="D80" s="4">
         <f>+D27-C27</f>
         <v>6283034</v>
@@ -2130,14 +2129,14 @@
         <f>+F27-E27</f>
         <v>-8524188</v>
       </c>
-      <c r="G80" s="27"/>
+      <c r="G80" s="12"/>
     </row>
     <row r="81" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A81" s="21"/>
-      <c r="B81" s="19" t="s">
+      <c r="A81" s="11"/>
+      <c r="B81" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="C81" s="20"/>
+      <c r="C81" s="15"/>
       <c r="D81" s="4">
         <f>+D29-C29</f>
         <v>-831606</v>
@@ -2150,16 +2149,16 @@
         <f>+F29-E29</f>
         <v>-935165</v>
       </c>
-      <c r="G81" s="27"/>
+      <c r="G81" s="12"/>
     </row>
     <row r="82" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A82" s="21" t="s">
+      <c r="A82" s="11" t="s">
         <v>81</v>
       </c>
-      <c r="B82" s="19" t="s">
+      <c r="B82" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="C82" s="20"/>
+      <c r="C82" s="15"/>
       <c r="D82" s="4">
         <f t="shared" ref="D82:F84" si="14">+D31-C31</f>
         <v>0</v>
@@ -2172,14 +2171,14 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="G82" s="27"/>
+      <c r="G82" s="12"/>
     </row>
     <row r="83" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A83" s="21"/>
-      <c r="B83" s="19" t="s">
+      <c r="A83" s="11"/>
+      <c r="B83" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="C83" s="20"/>
+      <c r="C83" s="15"/>
       <c r="D83" s="4">
         <f t="shared" si="14"/>
         <v>0</v>
@@ -2192,14 +2191,14 @@
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="G83" s="27"/>
+      <c r="G83" s="12"/>
     </row>
     <row r="84" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A84" s="21"/>
-      <c r="B84" s="19" t="s">
+      <c r="A84" s="11"/>
+      <c r="B84" s="14" t="s">
         <v>95</v>
       </c>
-      <c r="C84" s="20"/>
+      <c r="C84" s="15"/>
       <c r="D84" s="4">
         <f t="shared" si="14"/>
         <v>-55482500</v>
@@ -2212,14 +2211,14 @@
         <f t="shared" si="14"/>
         <v>101454998</v>
       </c>
-      <c r="G84" s="27"/>
+      <c r="G84" s="12"/>
     </row>
     <row r="85" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A85" s="21"/>
-      <c r="B85" s="19" t="s">
+      <c r="A85" s="11"/>
+      <c r="B85" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="C85" s="20"/>
+      <c r="C85" s="15"/>
       <c r="D85" s="4">
         <f>+D34+D35-C34-C35</f>
         <v>0</v>
@@ -2232,14 +2231,14 @@
         <f>+F34+F35-E34-E35</f>
         <v>0</v>
       </c>
-      <c r="G85" s="27"/>
+      <c r="G85" s="12"/>
     </row>
     <row r="86" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A86" s="21"/>
-      <c r="B86" s="19" t="s">
+      <c r="A86" s="11"/>
+      <c r="B86" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="C86" s="20"/>
+      <c r="C86" s="15"/>
       <c r="D86" s="4">
         <f>+D37-C37</f>
         <v>1324193</v>
@@ -2252,14 +2251,14 @@
         <f>+F37-E37</f>
         <v>11288640</v>
       </c>
-      <c r="G86" s="27"/>
+      <c r="G86" s="12"/>
     </row>
     <row r="87" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A87" s="3"/>
-      <c r="B87" s="11" t="s">
+      <c r="B87" s="22" t="s">
         <v>106</v>
       </c>
-      <c r="C87" s="12"/>
+      <c r="C87" s="23"/>
       <c r="D87" s="5">
         <f>SUM(D68:D86)</f>
         <v>-74636645</v>
@@ -2278,10 +2277,10 @@
       <c r="A88" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="B88" s="19" t="s">
+      <c r="B88" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="C88" s="20"/>
+      <c r="C88" s="15"/>
       <c r="D88" s="4">
         <f>+C14+C16-D14-D16-D63</f>
         <v>-9263629</v>
@@ -2299,13 +2298,13 @@
       </c>
     </row>
     <row r="89" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A89" s="21" t="s">
+      <c r="A89" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="B89" s="19" t="s">
+      <c r="B89" s="14" t="s">
         <v>73</v>
       </c>
-      <c r="C89" s="20"/>
+      <c r="C89" s="15"/>
       <c r="D89" s="4">
         <f>+C13-D13</f>
         <v>0</v>
@@ -2321,11 +2320,11 @@
       <c r="G89" s="3"/>
     </row>
     <row r="90" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A90" s="21"/>
-      <c r="B90" s="19" t="s">
+      <c r="A90" s="11"/>
+      <c r="B90" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="C90" s="20"/>
+      <c r="C90" s="15"/>
       <c r="D90" s="4">
         <f>+C15-D15</f>
         <v>0</v>
@@ -2341,11 +2340,11 @@
       <c r="G90" s="3"/>
     </row>
     <row r="91" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A91" s="21"/>
-      <c r="B91" s="19" t="s">
+      <c r="A91" s="11"/>
+      <c r="B91" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="C91" s="20"/>
+      <c r="C91" s="15"/>
       <c r="D91" s="4">
         <f t="shared" ref="D91:F95" si="15">+C17-D17</f>
         <v>0</v>
@@ -2361,11 +2360,11 @@
       <c r="G91" s="3"/>
     </row>
     <row r="92" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A92" s="21"/>
-      <c r="B92" s="19" t="s">
+      <c r="A92" s="11"/>
+      <c r="B92" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="C92" s="20"/>
+      <c r="C92" s="15"/>
       <c r="D92" s="4">
         <f t="shared" si="15"/>
         <v>0</v>
@@ -2381,11 +2380,11 @@
       <c r="G92" s="3"/>
     </row>
     <row r="93" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A93" s="21"/>
-      <c r="B93" s="19" t="s">
+      <c r="A93" s="11"/>
+      <c r="B93" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="C93" s="20"/>
+      <c r="C93" s="15"/>
       <c r="D93" s="4">
         <f t="shared" si="15"/>
         <v>0</v>
@@ -2401,11 +2400,11 @@
       <c r="G93" s="3"/>
     </row>
     <row r="94" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A94" s="21"/>
-      <c r="B94" s="19" t="s">
+      <c r="A94" s="11"/>
+      <c r="B94" s="14" t="s">
         <v>78</v>
       </c>
-      <c r="C94" s="20"/>
+      <c r="C94" s="15"/>
       <c r="D94" s="4">
         <f t="shared" si="15"/>
         <v>0</v>
@@ -2421,11 +2420,11 @@
       <c r="G94" s="3"/>
     </row>
     <row r="95" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A95" s="21"/>
-      <c r="B95" s="19" t="s">
+      <c r="A95" s="11"/>
+      <c r="B95" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="C95" s="20"/>
+      <c r="C95" s="15"/>
       <c r="D95" s="4">
         <f t="shared" si="15"/>
         <v>0</v>
@@ -2442,10 +2441,10 @@
     </row>
     <row r="96" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A96" s="3"/>
-      <c r="B96" s="11" t="s">
+      <c r="B96" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="C96" s="12"/>
+      <c r="C96" s="23"/>
       <c r="D96" s="5">
         <f>SUM(D88:D95)</f>
         <v>-9263629</v>
@@ -2461,13 +2460,13 @@
       <c r="G96" s="3"/>
     </row>
     <row r="97" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A97" s="27" t="s">
+      <c r="A97" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="B97" s="13" t="s">
+      <c r="B97" s="16" t="s">
         <v>83</v>
       </c>
-      <c r="C97" s="14"/>
+      <c r="C97" s="17"/>
       <c r="D97" s="4">
         <f>+D28-C28</f>
         <v>0</v>
@@ -2483,11 +2482,11 @@
       <c r="G97" s="3"/>
     </row>
     <row r="98" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A98" s="27"/>
-      <c r="B98" s="13" t="s">
+      <c r="A98" s="12"/>
+      <c r="B98" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="C98" s="14"/>
+      <c r="C98" s="17"/>
       <c r="D98" s="4">
         <f>+D36-C36</f>
         <v>103658589</v>
@@ -2503,13 +2502,13 @@
       <c r="G98" s="3"/>
     </row>
     <row r="99" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A99" s="25" t="s">
+      <c r="A99" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="B99" s="13" t="s">
+      <c r="B99" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="C99" s="14"/>
+      <c r="C99" s="17"/>
       <c r="D99" s="4">
         <f t="shared" ref="D99:F100" si="16">+D40-C40</f>
         <v>0</v>
@@ -2525,11 +2524,11 @@
       <c r="G99" s="3"/>
     </row>
     <row r="100" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A100" s="25"/>
-      <c r="B100" s="13" t="s">
+      <c r="A100" s="13"/>
+      <c r="B100" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="C100" s="14"/>
+      <c r="C100" s="17"/>
       <c r="D100" s="4">
         <f t="shared" si="16"/>
         <v>0</v>
@@ -2546,10 +2545,10 @@
     </row>
     <row r="101" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A101" s="6"/>
-      <c r="B101" s="17" t="s">
+      <c r="B101" s="26" t="s">
         <v>105</v>
       </c>
-      <c r="C101" s="18"/>
+      <c r="C101" s="27"/>
       <c r="D101" s="4">
         <f>+C42+D61-D42</f>
         <v>0</v>
@@ -2570,10 +2569,10 @@
       <c r="A102" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="B102" s="17" t="s">
+      <c r="B102" s="26" t="s">
         <v>89</v>
       </c>
-      <c r="C102" s="18"/>
+      <c r="C102" s="27"/>
       <c r="D102" s="4">
         <f>-D58</f>
         <v>-6052503</v>
@@ -2592,10 +2591,10 @@
       <c r="A103" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="B103" s="17" t="s">
+      <c r="B103" s="26" t="s">
         <v>92</v>
       </c>
-      <c r="C103" s="18"/>
+      <c r="C103" s="27"/>
       <c r="D103" s="4">
         <f>+D57</f>
         <v>481784</v>
@@ -2612,10 +2611,10 @@
     </row>
     <row r="104" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A104" s="6"/>
-      <c r="B104" s="11" t="s">
+      <c r="B104" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="C104" s="12"/>
+      <c r="C104" s="23"/>
       <c r="D104" s="5">
         <f>SUM(D97:D103)</f>
         <v>98087870</v>
@@ -2637,10 +2636,10 @@
     </row>
     <row r="106" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A106" s="6"/>
-      <c r="B106" s="11" t="s">
+      <c r="B106" s="22" t="s">
         <v>104</v>
       </c>
-      <c r="C106" s="12"/>
+      <c r="C106" s="23"/>
       <c r="D106" s="5">
         <f>+D87+D96+D104</f>
         <v>14187596</v>
@@ -2655,10 +2654,10 @@
       </c>
     </row>
     <row r="107" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B107" s="13" t="s">
+      <c r="B107" s="16" t="s">
         <v>93</v>
       </c>
-      <c r="C107" s="14"/>
+      <c r="C107" s="17"/>
       <c r="D107" s="4">
         <f>+C6</f>
         <v>61719652</v>
@@ -2673,10 +2672,10 @@
       </c>
     </row>
     <row r="108" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B108" s="15" t="s">
+      <c r="B108" s="18" t="s">
         <v>94</v>
       </c>
-      <c r="C108" s="16"/>
+      <c r="C108" s="19"/>
       <c r="D108" s="5">
         <f>SUM(D106:D107)</f>
         <v>75907248</v>
@@ -2707,62 +2706,27 @@
     </row>
   </sheetData>
   <mergeCells count="109">
-    <mergeCell ref="A68:A71"/>
-    <mergeCell ref="G78:G86"/>
-    <mergeCell ref="A97:A98"/>
-    <mergeCell ref="A99:A100"/>
-    <mergeCell ref="A72:A74"/>
-    <mergeCell ref="A75:A77"/>
-    <mergeCell ref="A78:A81"/>
-    <mergeCell ref="A89:A95"/>
-    <mergeCell ref="A82:A86"/>
-    <mergeCell ref="B72:C72"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="B74:C74"/>
-    <mergeCell ref="B75:C75"/>
-    <mergeCell ref="B76:C76"/>
-    <mergeCell ref="B77:C77"/>
-    <mergeCell ref="B78:C78"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A34:B34"/>
-    <mergeCell ref="A35:B35"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="A44:B44"/>
-    <mergeCell ref="A48:B48"/>
-    <mergeCell ref="A45:B45"/>
-    <mergeCell ref="A46:B46"/>
-    <mergeCell ref="A47:B47"/>
-    <mergeCell ref="A36:B36"/>
-    <mergeCell ref="A37:B37"/>
-    <mergeCell ref="A38:B38"/>
-    <mergeCell ref="A39:B39"/>
-    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="B104:C104"/>
+    <mergeCell ref="B106:C106"/>
+    <mergeCell ref="B107:C107"/>
+    <mergeCell ref="B108:C108"/>
+    <mergeCell ref="B99:C99"/>
+    <mergeCell ref="B100:C100"/>
+    <mergeCell ref="B101:C101"/>
+    <mergeCell ref="B102:C102"/>
+    <mergeCell ref="B103:C103"/>
+    <mergeCell ref="B82:C82"/>
+    <mergeCell ref="B83:C83"/>
+    <mergeCell ref="B94:C94"/>
+    <mergeCell ref="B95:C95"/>
+    <mergeCell ref="B96:C96"/>
+    <mergeCell ref="B97:C97"/>
+    <mergeCell ref="B98:C98"/>
+    <mergeCell ref="B89:C89"/>
+    <mergeCell ref="B90:C90"/>
+    <mergeCell ref="B91:C91"/>
+    <mergeCell ref="B92:C92"/>
+    <mergeCell ref="B93:C93"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="B68:C68"/>
     <mergeCell ref="B69:C69"/>
@@ -2787,6 +2751,62 @@
     <mergeCell ref="A41:B41"/>
     <mergeCell ref="A42:B42"/>
     <mergeCell ref="A43:B43"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="A45:B45"/>
+    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A36:B36"/>
+    <mergeCell ref="A37:B37"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A33:B33"/>
+    <mergeCell ref="A34:B34"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="A68:A71"/>
+    <mergeCell ref="G78:G86"/>
+    <mergeCell ref="A97:A98"/>
+    <mergeCell ref="A99:A100"/>
+    <mergeCell ref="A72:A74"/>
+    <mergeCell ref="A75:A77"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="A89:A95"/>
+    <mergeCell ref="A82:A86"/>
+    <mergeCell ref="B72:C72"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="B74:C74"/>
+    <mergeCell ref="B75:C75"/>
+    <mergeCell ref="B76:C76"/>
+    <mergeCell ref="B77:C77"/>
+    <mergeCell ref="B78:C78"/>
     <mergeCell ref="B84:C84"/>
     <mergeCell ref="B85:C85"/>
     <mergeCell ref="B86:C86"/>
@@ -2795,27 +2815,6 @@
     <mergeCell ref="B79:C79"/>
     <mergeCell ref="B80:C80"/>
     <mergeCell ref="B81:C81"/>
-    <mergeCell ref="B82:C82"/>
-    <mergeCell ref="B83:C83"/>
-    <mergeCell ref="B94:C94"/>
-    <mergeCell ref="B95:C95"/>
-    <mergeCell ref="B96:C96"/>
-    <mergeCell ref="B97:C97"/>
-    <mergeCell ref="B98:C98"/>
-    <mergeCell ref="B89:C89"/>
-    <mergeCell ref="B90:C90"/>
-    <mergeCell ref="B91:C91"/>
-    <mergeCell ref="B92:C92"/>
-    <mergeCell ref="B93:C93"/>
-    <mergeCell ref="B104:C104"/>
-    <mergeCell ref="B106:C106"/>
-    <mergeCell ref="B107:C107"/>
-    <mergeCell ref="B108:C108"/>
-    <mergeCell ref="B99:C99"/>
-    <mergeCell ref="B100:C100"/>
-    <mergeCell ref="B101:C101"/>
-    <mergeCell ref="B102:C102"/>
-    <mergeCell ref="B103:C103"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>

<commit_message>
March 3 2025 V1
</commit_message>
<xml_diff>
--- a/_downloads/219fb1d9309965b5498bc9255adc60a7/Ejemplo Flujo de Efectivo H&M.xlsx
+++ b/_downloads/219fb1d9309965b5498bc9255adc60a7/Ejemplo Flujo de Efectivo H&M.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24729"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\UNAL\ADMINISTRACIÓN FINANCIERA\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E40B89F2-2167-4869-9302-9DBAD1069848}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C251891-E499-4104-83C0-7F021B862859}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{96756974-1267-4C41-A3A6-DE3697CF134B}"/>
   </bookViews>
@@ -348,9 +348,6 @@
     <t>+ Depreciación y Amortización</t>
   </si>
   <si>
-    <t>Ganancias acumuladas anteriores + Utilidad Neta actual - Ganancias acumuladas actuales</t>
-  </si>
-  <si>
     <t>Δ CAPEX (Capital Expenditure)</t>
   </si>
   <si>
@@ -370,6 +367,9 @@
   </si>
   <si>
     <t>Efectivo generado por Operación - EGO (a)</t>
+  </si>
+  <si>
+    <t>Ganancias acumuladas anteriores + Utilidad Neta actual - Ganancias acumuladas actuales - Aumentos Reservas u Otras Reservas período actual</t>
   </si>
 </sst>
 </file>
@@ -528,6 +528,12 @@
     <xf numFmtId="165" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -545,12 +551,6 @@
     </xf>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -583,9 +583,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -623,7 +623,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -729,7 +729,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -871,7 +871,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -907,7 +907,7 @@
     </row>
     <row r="5" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A5" s="11"/>
-      <c r="B5" s="21"/>
+      <c r="B5" s="23"/>
       <c r="C5" s="2">
         <v>2017</v>
       </c>
@@ -922,10 +922,10 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="17"/>
+      <c r="B6" s="19"/>
       <c r="C6" s="4">
         <v>61719652</v>
       </c>
@@ -940,10 +940,10 @@
       </c>
     </row>
     <row r="7" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="17"/>
+      <c r="B7" s="19"/>
       <c r="C7" s="4">
         <v>16010669</v>
       </c>
@@ -958,10 +958,10 @@
       </c>
     </row>
     <row r="8" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="17"/>
+      <c r="B8" s="19"/>
       <c r="C8" s="4">
         <v>41791255</v>
       </c>
@@ -976,10 +976,10 @@
       </c>
     </row>
     <row r="9" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="17"/>
+      <c r="B9" s="19"/>
       <c r="C9" s="4">
         <v>1485552</v>
       </c>
@@ -990,20 +990,20 @@
       <c r="F9" s="4"/>
     </row>
     <row r="10" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="17"/>
+      <c r="B10" s="19"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
     </row>
     <row r="11" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="16" t="s">
+      <c r="A11" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="17"/>
+      <c r="B11" s="19"/>
       <c r="C11" s="4">
         <v>2669096</v>
       </c>
@@ -1018,10 +1018,10 @@
       </c>
     </row>
     <row r="12" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A12" s="18" t="s">
+      <c r="A12" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="19"/>
+      <c r="B12" s="21"/>
       <c r="C12" s="5">
         <f>SUM(C6:C11)</f>
         <v>123676224</v>
@@ -1040,20 +1040,20 @@
       </c>
     </row>
     <row r="13" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="17"/>
+      <c r="B13" s="19"/>
       <c r="C13" s="4"/>
       <c r="D13" s="4"/>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
     </row>
     <row r="14" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="17"/>
+      <c r="B14" s="19"/>
       <c r="C14" s="4">
         <v>57777446</v>
       </c>
@@ -1068,50 +1068,50 @@
       </c>
     </row>
     <row r="15" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A15" s="16" t="s">
+      <c r="A15" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="17"/>
+      <c r="B15" s="19"/>
       <c r="C15" s="4"/>
       <c r="D15" s="4"/>
       <c r="E15" s="4"/>
       <c r="F15" s="4"/>
     </row>
     <row r="16" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="17"/>
+      <c r="B16" s="19"/>
       <c r="C16" s="4"/>
       <c r="D16" s="4"/>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
     </row>
     <row r="17" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A17" s="16" t="s">
+      <c r="A17" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="B17" s="17"/>
+      <c r="B17" s="19"/>
       <c r="C17" s="4"/>
       <c r="D17" s="4"/>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
     </row>
     <row r="18" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A18" s="16" t="s">
+      <c r="A18" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="17"/>
+      <c r="B18" s="19"/>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
     </row>
     <row r="19" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A19" s="16" t="s">
+      <c r="A19" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="B19" s="17"/>
+      <c r="B19" s="19"/>
       <c r="C19" s="4"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4">
@@ -1122,30 +1122,30 @@
       </c>
     </row>
     <row r="20" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A20" s="16" t="s">
+      <c r="A20" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="B20" s="17"/>
+      <c r="B20" s="19"/>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
     </row>
     <row r="21" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A21" s="16" t="s">
+      <c r="A21" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="B21" s="17"/>
+      <c r="B21" s="19"/>
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
       <c r="E21" s="4"/>
       <c r="F21" s="4"/>
     </row>
     <row r="22" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="18" t="s">
+      <c r="A22" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="19"/>
+      <c r="B22" s="21"/>
       <c r="C22" s="5">
         <f>SUM(C13:C21)</f>
         <v>57777446</v>
@@ -1164,10 +1164,10 @@
       </c>
     </row>
     <row r="23" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A23" s="18" t="s">
+      <c r="A23" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="B23" s="19"/>
+      <c r="B23" s="21"/>
       <c r="C23" s="5">
         <f>+C12+C22</f>
         <v>181453670</v>
@@ -1186,10 +1186,10 @@
       </c>
     </row>
     <row r="24" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A24" s="16" t="s">
+      <c r="A24" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="B24" s="17"/>
+      <c r="B24" s="19"/>
       <c r="C24" s="4">
         <v>920670</v>
       </c>
@@ -1204,10 +1204,10 @@
       </c>
     </row>
     <row r="25" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A25" s="16" t="s">
+      <c r="A25" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="17"/>
+      <c r="B25" s="19"/>
       <c r="C25" s="4">
         <v>610000</v>
       </c>
@@ -1218,10 +1218,10 @@
       <c r="F25" s="4"/>
     </row>
     <row r="26" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A26" s="16" t="s">
+      <c r="A26" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="B26" s="17"/>
+      <c r="B26" s="19"/>
       <c r="C26" s="4">
         <v>116865783</v>
       </c>
@@ -1236,10 +1236,10 @@
       </c>
     </row>
     <row r="27" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A27" s="16" t="s">
+      <c r="A27" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B27" s="17"/>
+      <c r="B27" s="19"/>
       <c r="C27" s="4">
         <v>588184</v>
       </c>
@@ -1254,10 +1254,10 @@
       </c>
     </row>
     <row r="28" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A28" s="16" t="s">
+      <c r="A28" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="B28" s="17"/>
+      <c r="B28" s="19"/>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
       <c r="E28" s="4">
@@ -1268,10 +1268,10 @@
       </c>
     </row>
     <row r="29" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A29" s="16" t="s">
+      <c r="A29" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="B29" s="17"/>
+      <c r="B29" s="19"/>
       <c r="C29" s="4">
         <v>831606</v>
       </c>
@@ -1284,10 +1284,10 @@
       </c>
     </row>
     <row r="30" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A30" s="18" t="s">
+      <c r="A30" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="B30" s="19"/>
+      <c r="B30" s="21"/>
       <c r="C30" s="5">
         <f>SUM(C24:C29)</f>
         <v>119816243</v>
@@ -1306,30 +1306,30 @@
       </c>
     </row>
     <row r="31" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A31" s="16" t="s">
+      <c r="A31" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="B31" s="17"/>
+      <c r="B31" s="19"/>
       <c r="C31" s="4"/>
       <c r="D31" s="4"/>
       <c r="E31" s="4"/>
       <c r="F31" s="4"/>
     </row>
     <row r="32" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A32" s="16" t="s">
+      <c r="A32" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="B32" s="17"/>
+      <c r="B32" s="19"/>
       <c r="C32" s="4"/>
       <c r="D32" s="4"/>
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
     </row>
     <row r="33" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A33" s="16" t="s">
+      <c r="A33" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="B33" s="17"/>
+      <c r="B33" s="19"/>
       <c r="C33" s="4">
         <v>55482500</v>
       </c>
@@ -1342,30 +1342,30 @@
       </c>
     </row>
     <row r="34" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A34" s="16" t="s">
+      <c r="A34" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="B34" s="17"/>
+      <c r="B34" s="19"/>
       <c r="C34" s="4"/>
       <c r="D34" s="4"/>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
     </row>
     <row r="35" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A35" s="16" t="s">
+      <c r="A35" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="B35" s="17"/>
+      <c r="B35" s="19"/>
       <c r="C35" s="4"/>
       <c r="D35" s="4"/>
       <c r="E35" s="4"/>
       <c r="F35" s="4"/>
     </row>
     <row r="36" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A36" s="16" t="s">
+      <c r="A36" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="B36" s="17"/>
+      <c r="B36" s="19"/>
       <c r="C36" s="4"/>
       <c r="D36" s="4">
         <v>103658589</v>
@@ -1378,10 +1378,10 @@
       </c>
     </row>
     <row r="37" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A37" s="16" t="s">
+      <c r="A37" s="18" t="s">
         <v>34</v>
       </c>
-      <c r="B37" s="17"/>
+      <c r="B37" s="19"/>
       <c r="C37" s="4"/>
       <c r="D37" s="4">
         <v>1324193</v>
@@ -1394,10 +1394,10 @@
       </c>
     </row>
     <row r="38" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A38" s="18" t="s">
+      <c r="A38" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="B38" s="19"/>
+      <c r="B38" s="21"/>
       <c r="C38" s="5">
         <f>SUM(C31:C37)</f>
         <v>55482500</v>
@@ -1416,10 +1416,10 @@
       </c>
     </row>
     <row r="39" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A39" s="18" t="s">
+      <c r="A39" s="20" t="s">
         <v>36</v>
       </c>
-      <c r="B39" s="19"/>
+      <c r="B39" s="21"/>
       <c r="C39" s="5">
         <f>+C30+C38</f>
         <v>175298743</v>
@@ -1438,10 +1438,10 @@
       </c>
     </row>
     <row r="40" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A40" s="16" t="s">
+      <c r="A40" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="B40" s="17"/>
+      <c r="B40" s="19"/>
       <c r="C40" s="4">
         <v>2521750</v>
       </c>
@@ -1456,10 +1456,10 @@
       </c>
     </row>
     <row r="41" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A41" s="16" t="s">
+      <c r="A41" s="18" t="s">
         <v>38</v>
       </c>
-      <c r="B41" s="17"/>
+      <c r="B41" s="19"/>
       <c r="C41" s="4">
         <v>22065750</v>
       </c>
@@ -1474,10 +1474,10 @@
       </c>
     </row>
     <row r="42" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A42" s="16" t="s">
+      <c r="A42" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="B42" s="17"/>
+      <c r="B42" s="19"/>
       <c r="C42" s="4">
         <v>-18432573</v>
       </c>
@@ -1492,10 +1492,10 @@
       </c>
     </row>
     <row r="43" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A43" s="18" t="s">
+      <c r="A43" s="20" t="s">
         <v>40</v>
       </c>
-      <c r="B43" s="19"/>
+      <c r="B43" s="21"/>
       <c r="C43" s="5">
         <f>SUM(C40:C42)</f>
         <v>6154927</v>
@@ -1514,10 +1514,10 @@
       </c>
     </row>
     <row r="44" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A44" s="18" t="s">
+      <c r="A44" s="20" t="s">
         <v>41</v>
       </c>
-      <c r="B44" s="19"/>
+      <c r="B44" s="21"/>
       <c r="C44" s="5">
         <f>+C39+C43</f>
         <v>181453670</v>
@@ -1545,7 +1545,7 @@
     </row>
     <row r="47" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A47" s="13"/>
-      <c r="B47" s="20"/>
+      <c r="B47" s="22"/>
       <c r="C47" s="2">
         <v>2017</v>
       </c>
@@ -1560,10 +1560,10 @@
       </c>
     </row>
     <row r="48" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A48" s="16" t="s">
+      <c r="A48" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="B48" s="17"/>
+      <c r="B48" s="19"/>
       <c r="C48" s="4">
         <v>95221493</v>
       </c>
@@ -1578,10 +1578,10 @@
       </c>
     </row>
     <row r="49" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A49" s="16" t="s">
+      <c r="A49" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="B49" s="17"/>
+      <c r="B49" s="19"/>
       <c r="C49" s="4">
         <v>48837338</v>
       </c>
@@ -1596,10 +1596,10 @@
       </c>
     </row>
     <row r="50" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A50" s="18" t="s">
+      <c r="A50" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="B50" s="19"/>
+      <c r="B50" s="21"/>
       <c r="C50" s="5">
         <f>+C48-C49</f>
         <v>46384155</v>
@@ -1618,10 +1618,10 @@
       </c>
     </row>
     <row r="51" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A51" s="16" t="s">
+      <c r="A51" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="B51" s="17"/>
+      <c r="B51" s="19"/>
       <c r="C51" s="4">
         <v>5388102</v>
       </c>
@@ -1630,10 +1630,10 @@
       <c r="F51" s="4"/>
     </row>
     <row r="52" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A52" s="16" t="s">
+      <c r="A52" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="B52" s="17"/>
+      <c r="B52" s="19"/>
       <c r="C52" s="4">
         <v>41445847</v>
       </c>
@@ -1646,10 +1646,10 @@
       </c>
     </row>
     <row r="53" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A53" s="16" t="s">
+      <c r="A53" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="B53" s="17"/>
+      <c r="B53" s="19"/>
       <c r="C53" s="4">
         <v>19209605</v>
       </c>
@@ -1664,10 +1664,10 @@
       </c>
     </row>
     <row r="54" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A54" s="16" t="s">
+      <c r="A54" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="B54" s="17"/>
+      <c r="B54" s="19"/>
       <c r="C54" s="4">
         <v>627842</v>
       </c>
@@ -1678,10 +1678,10 @@
       <c r="F54" s="4"/>
     </row>
     <row r="55" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A55" s="16" t="s">
+      <c r="A55" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="B55" s="17"/>
+      <c r="B55" s="19"/>
       <c r="C55" s="4"/>
       <c r="D55" s="4">
         <v>-3781821</v>
@@ -1694,10 +1694,10 @@
       </c>
     </row>
     <row r="56" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A56" s="18" t="s">
+      <c r="A56" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="B56" s="19"/>
+      <c r="B56" s="21"/>
       <c r="C56" s="5">
         <f>+C50+C51-C52-C53-C54+C55</f>
         <v>-9511037</v>
@@ -1717,10 +1717,10 @@
       <c r="G56" s="7"/>
     </row>
     <row r="57" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A57" s="16" t="s">
+      <c r="A57" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="B57" s="17"/>
+      <c r="B57" s="19"/>
       <c r="C57" s="4">
         <v>312884</v>
       </c>
@@ -1735,10 +1735,10 @@
       </c>
     </row>
     <row r="58" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A58" s="16" t="s">
+      <c r="A58" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="B58" s="17"/>
+      <c r="B58" s="19"/>
       <c r="C58" s="4">
         <v>7196584</v>
       </c>
@@ -1753,10 +1753,10 @@
       </c>
     </row>
     <row r="59" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A59" s="18" t="s">
+      <c r="A59" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="B59" s="19"/>
+      <c r="B59" s="21"/>
       <c r="C59" s="5">
         <f>+C56+C57-C58</f>
         <v>-16394737</v>
@@ -1775,10 +1775,10 @@
       </c>
     </row>
     <row r="60" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A60" s="16" t="s">
+      <c r="A60" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="B60" s="17"/>
+      <c r="B60" s="19"/>
       <c r="C60" s="4">
         <v>0</v>
       </c>
@@ -1793,10 +1793,10 @@
       </c>
     </row>
     <row r="61" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A61" s="18" t="s">
+      <c r="A61" s="20" t="s">
         <v>55</v>
       </c>
-      <c r="B61" s="19"/>
+      <c r="B61" s="21"/>
       <c r="C61" s="5">
         <f>+C59-C60</f>
         <v>-16394737</v>
@@ -1837,10 +1837,10 @@
       </c>
     </row>
     <row r="64" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A64" s="16" t="s">
+      <c r="A64" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="B64" s="17"/>
+      <c r="B64" s="19"/>
       <c r="C64" s="5">
         <f>+C56+C63</f>
         <v>-5628556</v>
@@ -1873,10 +1873,10 @@
     </row>
     <row r="68" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A68" s="11"/>
-      <c r="B68" s="22" t="s">
+      <c r="B68" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="C68" s="23"/>
+      <c r="C68" s="17"/>
       <c r="D68" s="4">
         <f>+D61</f>
         <v>-2861832</v>
@@ -2255,10 +2255,10 @@
     </row>
     <row r="87" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A87" s="3"/>
-      <c r="B87" s="22" t="s">
-        <v>106</v>
-      </c>
-      <c r="C87" s="23"/>
+      <c r="B87" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="C87" s="17"/>
       <c r="D87" s="5">
         <f>SUM(D68:D86)</f>
         <v>-74636645</v>
@@ -2275,7 +2275,7 @@
     </row>
     <row r="88" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A88" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B88" s="14" t="s">
         <v>71</v>
@@ -2294,7 +2294,7 @@
         <v>-24959140</v>
       </c>
       <c r="G88" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="89" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
@@ -2441,10 +2441,10 @@
     </row>
     <row r="96" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A96" s="3"/>
-      <c r="B96" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="C96" s="23"/>
+      <c r="B96" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="C96" s="17"/>
       <c r="D96" s="5">
         <f>SUM(D88:D95)</f>
         <v>-9263629</v>
@@ -2463,10 +2463,10 @@
       <c r="A97" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="B97" s="16" t="s">
+      <c r="B97" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="C97" s="17"/>
+      <c r="C97" s="19"/>
       <c r="D97" s="4">
         <f>+D28-C28</f>
         <v>0</v>
@@ -2483,10 +2483,10 @@
     </row>
     <row r="98" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A98" s="12"/>
-      <c r="B98" s="16" t="s">
+      <c r="B98" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="C98" s="17"/>
+      <c r="C98" s="19"/>
       <c r="D98" s="4">
         <f>+D36-C36</f>
         <v>103658589</v>
@@ -2505,10 +2505,10 @@
       <c r="A99" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="B99" s="16" t="s">
+      <c r="B99" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="C99" s="17"/>
+      <c r="C99" s="19"/>
       <c r="D99" s="4">
         <f t="shared" ref="D99:F100" si="16">+D40-C40</f>
         <v>0</v>
@@ -2525,10 +2525,10 @@
     </row>
     <row r="100" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A100" s="13"/>
-      <c r="B100" s="16" t="s">
+      <c r="B100" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="C100" s="17"/>
+      <c r="C100" s="19"/>
       <c r="D100" s="4">
         <f t="shared" si="16"/>
         <v>0</v>
@@ -2546,7 +2546,7 @@
     <row r="101" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A101" s="6"/>
       <c r="B101" s="26" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C101" s="27"/>
       <c r="D101" s="4">
@@ -2562,7 +2562,7 @@
         <v>0</v>
       </c>
       <c r="G101" s="3" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
     </row>
     <row r="102" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
@@ -2611,10 +2611,10 @@
     </row>
     <row r="104" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A104" s="6"/>
-      <c r="B104" s="22" t="s">
-        <v>103</v>
-      </c>
-      <c r="C104" s="23"/>
+      <c r="B104" s="16" t="s">
+        <v>102</v>
+      </c>
+      <c r="C104" s="17"/>
       <c r="D104" s="5">
         <f>SUM(D97:D103)</f>
         <v>98087870</v>
@@ -2636,10 +2636,10 @@
     </row>
     <row r="106" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A106" s="6"/>
-      <c r="B106" s="22" t="s">
-        <v>104</v>
-      </c>
-      <c r="C106" s="23"/>
+      <c r="B106" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="C106" s="17"/>
       <c r="D106" s="5">
         <f>+D87+D96+D104</f>
         <v>14187596</v>
@@ -2654,10 +2654,10 @@
       </c>
     </row>
     <row r="107" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B107" s="16" t="s">
+      <c r="B107" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="C107" s="17"/>
+      <c r="C107" s="19"/>
       <c r="D107" s="4">
         <f>+C6</f>
         <v>61719652</v>
@@ -2672,10 +2672,10 @@
       </c>
     </row>
     <row r="108" spans="1:7" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="B108" s="18" t="s">
+      <c r="B108" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="C108" s="19"/>
+      <c r="C108" s="21"/>
       <c r="D108" s="5">
         <f>SUM(D106:D107)</f>
         <v>75907248</v>

</xml_diff>